<commit_message>
Refactor HTML structure and improve accessibility: remove inline styles for contrast button, adjust video width, and enhance label elements in feedback form; update CSS for video and high-contrast styles.
</commit_message>
<xml_diff>
--- a/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
+++ b/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="113">
   <si>
     <t xml:space="preserve">Web-fejlesztés kurzus beadandó feladata</t>
   </si>
@@ -197,7 +197,7 @@
     <t xml:space="preserve">Van olyan oldal, amelyben egy olyan űrlap található, amely tartalmaz legalább egy szövegmezőt (text), egy szövegterületet (textarea),legalább 2 választókapcsolót (radio), legalább 1 jelölőnégyzetet (checkbox), valamint egy elküldés (submit) gombot. </t>
   </si>
   <si>
-    <t xml:space="preserve">írd ide , hogy melyik oldal</t>
+    <t xml:space="preserve">extras.html</t>
   </si>
   <si>
     <r>
@@ -224,7 +224,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">írd ide hogy melyik oldalon van, és mit csinál a script</t>
+    <t xml:space="preserve">mindegyik oldalon, a high contrast gomb</t>
   </si>
   <si>
     <r>
@@ -614,6 +614,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Gameplay video van az oldalon, nem tudom hogy ide kötelező-e narrátor, de megpróbálok bele rakni valamit</t>
+  </si>
+  <si>
     <t xml:space="preserve">Az oldal nyelve mindegyik oldalon beállításra került. Ahol az alapértelmezett nyelvtől eltérő szöveg is van az oldalon, az el van látva a megfelelő nyelvkóddal.</t>
   </si>
   <si>
@@ -633,6 +636,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mindegyik beadott oldal a HTML5 szabvány szerint készült és valid a https://validator.w3.org/ oldal szerint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mindegyik oldal valid a validator szerint</t>
   </si>
   <si>
     <r>
@@ -657,6 +663,9 @@
       </rPr>
       <t xml:space="preserve">Amennyiben a Bootstrap keretrendszer lett használva, a saját készítésű stílusok megfelelően elkülönülnek a Bootstrap stílusállományaitól.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">style.css</t>
   </si>
   <si>
     <t xml:space="preserve">Statisztika (hallgatói értékelés)</t>
@@ -1947,7 +1956,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.888888888888889</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.857142857142857</c:v>
@@ -1959,13 +1968,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="96790786"/>
-        <c:axId val="59539527"/>
+        <c:axId val="27720609"/>
+        <c:axId val="27951075"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="96790786"/>
+        <c:axId val="27720609"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2004,7 +2013,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59539527"/>
+        <c:crossAx val="27951075"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2012,7 +2021,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59539527"/>
+        <c:axId val="27951075"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2057,7 +2066,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96790786"/>
+        <c:crossAx val="27720609"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2260,7 +2269,7 @@
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>6</c:v>
@@ -2363,7 +2372,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1</c:v>
@@ -2377,11 +2386,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="7767783"/>
-        <c:axId val="79327621"/>
+        <c:axId val="88448388"/>
+        <c:axId val="43554698"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="7767783"/>
+        <c:axId val="88448388"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2415,7 +2424,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79327621"/>
+        <c:crossAx val="43554698"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2423,7 +2432,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79327621"/>
+        <c:axId val="43554698"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -2458,7 +2467,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7767783"/>
+        <c:crossAx val="88448388"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -2669,13 +2678,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="88008957"/>
-        <c:axId val="91090096"/>
+        <c:axId val="30567362"/>
+        <c:axId val="90971128"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="88008957"/>
+        <c:axId val="30567362"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2714,7 +2723,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91090096"/>
+        <c:crossAx val="90971128"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2722,7 +2731,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91090096"/>
+        <c:axId val="90971128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2767,7 +2776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88008957"/>
+        <c:crossAx val="30567362"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3087,11 +3096,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="21212877"/>
-        <c:axId val="48094281"/>
+        <c:axId val="27032562"/>
+        <c:axId val="90223683"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="21212877"/>
+        <c:axId val="27032562"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3125,7 +3134,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48094281"/>
+        <c:crossAx val="90223683"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3133,7 +3142,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48094281"/>
+        <c:axId val="90223683"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -3168,7 +3177,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21212877"/>
+        <c:crossAx val="27032562"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -3297,9 +3306,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>25200</xdr:colOff>
+      <xdr:colOff>24840</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>149400</xdr:rowOff>
+      <xdr:rowOff>149040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3308,7 +3317,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6618600" cy="4875480"/>
+        <a:ext cx="6618240" cy="4875120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3327,9 +3336,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884880</xdr:colOff>
+      <xdr:colOff>884520</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>25200</xdr:rowOff>
+      <xdr:rowOff>24840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3338,7 +3347,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5003280" cy="2770560"/>
+        <a:ext cx="5002920" cy="2770200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3362,9 +3371,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>34920</xdr:colOff>
+      <xdr:colOff>34560</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>149400</xdr:rowOff>
+      <xdr:rowOff>149040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3373,7 +3382,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6628320" cy="4875480"/>
+        <a:ext cx="6627960" cy="4875120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3392,9 +3401,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884880</xdr:colOff>
+      <xdr:colOff>884520</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>25200</xdr:rowOff>
+      <xdr:rowOff>24840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3403,7 +3412,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5003280" cy="2770560"/>
+        <a:ext cx="5002920" cy="2770200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3824,7 +3833,7 @@
       <c r="C15" s="13"/>
       <c r="D15" s="16" t="n">
         <f aca="false">SUM(Irányelvek!J2:J48)</f>
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="17" t="str">
@@ -5096,7 +5105,9 @@
       <c r="C27" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="D27" s="45"/>
+      <c r="D27" s="45" t="n">
+        <v>1</v>
+      </c>
       <c r="E27" s="46"/>
       <c r="F27" s="45"/>
       <c r="G27" s="47"/>
@@ -5104,9 +5115,9 @@
       <c r="I27" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="J27" s="49" t="str">
+      <c r="J27" s="49" t="n">
         <f aca="false">IF(D27=1,I27,IF(H27=TRUE(),-5,""))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K27" s="50" t="str">
         <f aca="false">IF(F27=1,I27,IF(H27=TRUE(),-5,""))</f>
@@ -5114,7 +5125,7 @@
       </c>
       <c r="L27" s="49" t="n">
         <f aca="false">IF(J27=K27,0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5580,7 +5591,9 @@
         <v>87</v>
       </c>
       <c r="D41" s="45"/>
-      <c r="E41" s="87"/>
+      <c r="E41" s="87" t="s">
+        <v>88</v>
+      </c>
       <c r="F41" s="45"/>
       <c r="G41" s="88"/>
       <c r="H41" s="89"/>
@@ -5609,7 +5622,7 @@
         <v>81</v>
       </c>
       <c r="C42" s="63" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D42" s="64" t="n">
         <v>1</v>
@@ -5640,10 +5653,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="92" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C43" s="74" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D43" s="45" t="n">
         <v>1</v>
@@ -5677,10 +5690,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="93" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C44" s="58" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D44" s="45" t="n">
         <v>1</v>
@@ -5714,10 +5727,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="93" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C45" s="58" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D45" s="45" t="n">
         <v>1</v>
@@ -5751,10 +5764,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="93" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C46" s="58" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D46" s="45" t="n">
         <v>1</v>
@@ -5788,16 +5801,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="93" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C47" s="58" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D47" s="45" t="n">
         <v>1</v>
       </c>
       <c r="E47" s="53" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="F47" s="45"/>
       <c r="G47" s="94"/>
@@ -5827,16 +5840,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="93" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C48" s="58" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D48" s="45" t="n">
         <v>1</v>
       </c>
       <c r="E48" s="53" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="F48" s="45"/>
       <c r="G48" s="94"/>
@@ -5911,7 +5924,7 @@
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11"/>
       <c r="B1" s="95" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C1" s="95"/>
       <c r="D1" s="95"/>
@@ -5945,16 +5958,16 @@
       <c r="A2" s="11"/>
       <c r="B2" s="96"/>
       <c r="C2" s="97" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D2" s="97" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E2" s="97" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F2" s="97" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -6075,18 +6088,18 @@
       </c>
       <c r="C5" s="96" t="n">
         <f aca="false">COUNTIFS(Irányelvek!B4:B50,"="&amp;B5,Irányelvek!D4:D50,1)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="96" t="n">
         <f aca="false">E5-C5</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="99" t="n">
         <v>9</v>
       </c>
       <c r="F5" s="100" t="n">
         <f aca="false">C5/E5</f>
-        <v>0.888888888888889</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -6159,7 +6172,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11"/>
       <c r="B7" s="98" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C7" s="96" t="n">
         <f aca="false">COUNTIFS(Irányelvek!B6:B52,"="&amp;B7,Irányelvek!D6:D52,1)</f>
@@ -6203,15 +6216,15 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11"/>
       <c r="B8" s="101" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C8" s="102" t="n">
         <f aca="false">SUM(C3:C7)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="102" t="n">
         <f aca="false">SUM(D3:D7)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="102" t="n">
         <f aca="false">SUM(E3:E7)</f>
@@ -6219,7 +6232,7 @@
       </c>
       <c r="F8" s="100" t="n">
         <f aca="false">C8/E8</f>
-        <v>0.957446808510638</v>
+        <v>0.978723404255319</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
@@ -6748,7 +6761,7 @@
       <c r="D25" s="103"/>
       <c r="E25" s="103"/>
       <c r="F25" s="104" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G25" s="11"/>
       <c r="H25" s="11"/>
@@ -7516,7 +7529,7 @@
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11"/>
       <c r="B1" s="95" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C1" s="95"/>
       <c r="D1" s="95"/>
@@ -7550,16 +7563,16 @@
       <c r="A2" s="11"/>
       <c r="B2" s="96"/>
       <c r="C2" s="97" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D2" s="97" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E2" s="97" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F2" s="97" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -7765,7 +7778,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11"/>
       <c r="B7" s="98" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C7" s="96" t="n">
         <f aca="false">COUNTIFS(Irányelvek!B6:B52,"="&amp;B7,Irányelvek!F6:F52,1)</f>
@@ -7809,7 +7822,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11"/>
       <c r="B8" s="101" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C8" s="102" t="n">
         <f aca="false">SUM(C3:C7)</f>
@@ -8354,7 +8367,7 @@
       <c r="D25" s="103"/>
       <c r="E25" s="103"/>
       <c r="F25" s="104" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G25" s="11"/>
       <c r="H25" s="11"/>
@@ -9122,7 +9135,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="107" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C1" s="108"/>
       <c r="D1" s="108"/>
@@ -9143,7 +9156,7 @@
         <v>-100</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H3" s="1" t="n">
         <v>56</v>
@@ -9165,7 +9178,7 @@
         <v>50</v>
       </c>
       <c r="D4" s="56" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">H3/2</f>
@@ -9181,7 +9194,7 @@
         <v>63</v>
       </c>
       <c r="D5" s="56" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9193,7 +9206,7 @@
         <v>76</v>
       </c>
       <c r="D6" s="56" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9205,7 +9218,7 @@
         <v>89</v>
       </c>
       <c r="D7" s="56" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update video source and add narration transcript for gameplay video; modify Excel file
</commit_message>
<xml_diff>
--- a/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
+++ b/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
@@ -614,7 +614,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Gameplay video van az oldalon, nem tudom hogy ide kötelező-e narrátor, de megpróbálok bele rakni valamit</t>
+    <t xml:space="preserve">Gameplay video van az oldalon, nem tudom hogy ide kötelező-e narrátor, de próbáltam rakni bele</t>
   </si>
   <si>
     <t xml:space="preserve">Az oldal nyelve mindegyik oldalon beállításra került. Ahol az alapértelmezett nyelvtől eltérő szöveg is van az oldalon, az el van látva a megfelelő nyelvkóddal.</t>
@@ -1883,7 +1883,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4f81bd"/>
+              <a:srgbClr val="4F81BD"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -1959,7 +1959,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.857142857142857</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -1968,13 +1968,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="27720609"/>
-        <c:axId val="27951075"/>
+        <c:axId val="64889250"/>
+        <c:axId val="75166582"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="27720609"/>
+        <c:axId val="64889250"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2013,7 +2013,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27951075"/>
+        <c:crossAx val="75166582"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2021,7 +2021,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27951075"/>
+        <c:axId val="75166582"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2032,7 +2032,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="c1d1ec"/>
+                <a:srgbClr val="C1D1EC"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2066,13 +2066,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27720609"/>
+        <c:crossAx val="64889250"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
-          <a:srgbClr val="ffffff"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
         <a:ln w="0">
           <a:noFill/>
@@ -2120,11 +2120,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -2194,7 +2194,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4f81bd"/>
+              <a:srgbClr val="4F81BD"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -2272,7 +2272,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>6</c:v>
@@ -2297,7 +2297,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c0504d"/>
+              <a:srgbClr val="C0504D"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -2375,7 +2375,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2386,11 +2386,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="88448388"/>
-        <c:axId val="43554698"/>
+        <c:axId val="94826915"/>
+        <c:axId val="26523091"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88448388"/>
+        <c:axId val="94826915"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2424,7 +2424,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43554698"/>
+        <c:crossAx val="26523091"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2432,7 +2432,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43554698"/>
+        <c:axId val="26523091"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -2467,12 +2467,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88448388"/>
+        <c:crossAx val="94826915"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
-          <a:srgbClr val="ffffff"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
         <a:ln w="0">
           <a:noFill/>
@@ -2520,11 +2520,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -2593,7 +2593,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4f81bd"/>
+              <a:srgbClr val="4F81BD"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -2678,13 +2678,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="30567362"/>
-        <c:axId val="90971128"/>
+        <c:axId val="12785965"/>
+        <c:axId val="751057"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="30567362"/>
+        <c:axId val="12785965"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2723,7 +2723,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90971128"/>
+        <c:crossAx val="751057"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2731,7 +2731,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90971128"/>
+        <c:axId val="751057"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2742,7 +2742,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="c1d1ec"/>
+                <a:srgbClr val="C1D1EC"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2776,13 +2776,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30567362"/>
+        <c:crossAx val="12785965"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
-          <a:srgbClr val="ffffff"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
         <a:ln w="0">
           <a:noFill/>
@@ -2830,11 +2830,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -2904,7 +2904,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4f81bd"/>
+              <a:srgbClr val="4F81BD"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -3007,7 +3007,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c0504d"/>
+              <a:srgbClr val="C0504D"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -3096,11 +3096,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="27032562"/>
-        <c:axId val="90223683"/>
+        <c:axId val="79773851"/>
+        <c:axId val="23745984"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27032562"/>
+        <c:axId val="79773851"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3134,7 +3134,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90223683"/>
+        <c:crossAx val="23745984"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3142,7 +3142,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90223683"/>
+        <c:axId val="23745984"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -3177,12 +3177,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27032562"/>
+        <c:crossAx val="79773851"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
-          <a:srgbClr val="ffffff"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
         <a:ln w="0">
           <a:noFill/>
@@ -3230,16 +3230,880 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
   </c:spPr>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/ctrlProps/ctrlProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3306,9 +4170,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>24840</xdr:colOff>
+      <xdr:colOff>24480</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>149040</xdr:rowOff>
+      <xdr:rowOff>148680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3317,7 +4181,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6618240" cy="4875120"/>
+        <a:ext cx="6617880" cy="4874760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3336,9 +4200,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884520</xdr:colOff>
+      <xdr:colOff>884160</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>24840</xdr:rowOff>
+      <xdr:rowOff>24480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3347,7 +4211,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5002920" cy="2770200"/>
+        <a:ext cx="5002560" cy="2769840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3371,9 +4235,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>34560</xdr:colOff>
+      <xdr:colOff>34200</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>149040</xdr:rowOff>
+      <xdr:rowOff>148680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3382,7 +4246,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6627960" cy="4875120"/>
+        <a:ext cx="6627600" cy="4874760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3401,9 +4265,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884520</xdr:colOff>
+      <xdr:colOff>884160</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>24840</xdr:rowOff>
+      <xdr:rowOff>24480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3412,7 +4276,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5002920" cy="2770200"/>
+        <a:ext cx="5002560" cy="2769840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3433,34 +4297,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -3833,7 +4697,7 @@
       <c r="C15" s="13"/>
       <c r="D15" s="16" t="n">
         <f aca="false">SUM(Irányelvek!J2:J48)</f>
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="17" t="str">
@@ -5590,7 +6454,9 @@
       <c r="C41" s="86" t="s">
         <v>87</v>
       </c>
-      <c r="D41" s="45"/>
+      <c r="D41" s="45" t="n">
+        <v>1</v>
+      </c>
       <c r="E41" s="87" t="s">
         <v>88</v>
       </c>
@@ -5600,9 +6466,9 @@
       <c r="I41" s="90" t="n">
         <v>5</v>
       </c>
-      <c r="J41" s="49" t="str">
+      <c r="J41" s="49" t="n">
         <f aca="false">IF(D41=1,I41,IF(H41=TRUE(),-5,""))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="K41" s="50" t="str">
         <f aca="false">IF(F41=1,I41,IF(H41=TRUE(),-5,""))</f>
@@ -5610,7 +6476,7 @@
       </c>
       <c r="L41" s="56" t="n">
         <f aca="false">IF(J41=K41,0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" s="77" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6132,18 +6998,18 @@
       </c>
       <c r="C6" s="96" t="n">
         <f aca="false">COUNTIFS(Irányelvek!B5:B51,"="&amp;B6,Irányelvek!D5:D51,1)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="96" t="n">
         <f aca="false">E6-C6</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="99" t="n">
         <v>7</v>
       </c>
       <c r="F6" s="100" t="n">
         <f aca="false">C6/E6</f>
-        <v>0.857142857142857</v>
+        <v>1</v>
       </c>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
@@ -6220,11 +7086,11 @@
       </c>
       <c r="C8" s="102" t="n">
         <f aca="false">SUM(C3:C7)</f>
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="102" t="n">
         <f aca="false">SUM(D3:D7)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="102" t="n">
         <f aca="false">SUM(E3:E7)</f>
@@ -6232,7 +7098,7 @@
       </c>
       <c r="F8" s="100" t="n">
         <f aca="false">C8/E8</f>
-        <v>0.978723404255319</v>
+        <v>1</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>

</xml_diff>

<commit_message>
Add address file with project URL and update Excel guidelines
</commit_message>
<xml_diff>
--- a/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
+++ b/semester2/Web/assignment/phase2/webfejlesztes_iranyelvek_v202526_v1.xlsx
@@ -614,7 +614,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Gameplay video van az oldalon, nem tudom hogy ide kötelező-e narrátor, de próbáltam rakni bele</t>
+    <t xml:space="preserve">Gameplay video van az oldalon, raktam bele narrációt</t>
   </si>
   <si>
     <t xml:space="preserve">Az oldal nyelve mindegyik oldalon beállításra került. Ahol az alapértelmezett nyelvtől eltérő szöveg is van az oldalon, az el van látva a megfelelő nyelvkóddal.</t>
@@ -1968,13 +1968,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="64889250"/>
-        <c:axId val="75166582"/>
+        <c:axId val="22521073"/>
+        <c:axId val="6378568"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="64889250"/>
+        <c:axId val="22521073"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2013,7 +2013,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75166582"/>
+        <c:crossAx val="6378568"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2021,7 +2021,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75166582"/>
+        <c:axId val="6378568"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2066,7 +2066,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64889250"/>
+        <c:crossAx val="22521073"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2386,11 +2386,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="94826915"/>
-        <c:axId val="26523091"/>
+        <c:axId val="52056617"/>
+        <c:axId val="42533000"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94826915"/>
+        <c:axId val="52056617"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2424,7 +2424,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26523091"/>
+        <c:crossAx val="42533000"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2432,7 +2432,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26523091"/>
+        <c:axId val="42533000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -2467,7 +2467,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94826915"/>
+        <c:crossAx val="52056617"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -2678,13 +2678,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="12785965"/>
-        <c:axId val="751057"/>
+        <c:axId val="4377187"/>
+        <c:axId val="15028367"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="12785965"/>
+        <c:axId val="4377187"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2723,7 +2723,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="751057"/>
+        <c:crossAx val="15028367"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2731,7 +2731,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="751057"/>
+        <c:axId val="15028367"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2776,7 +2776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12785965"/>
+        <c:crossAx val="4377187"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3096,11 +3096,11 @@
         </c:ser>
         <c:gapWidth val="95"/>
         <c:overlap val="100"/>
-        <c:axId val="79773851"/>
-        <c:axId val="23745984"/>
+        <c:axId val="88892462"/>
+        <c:axId val="91149792"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="79773851"/>
+        <c:axId val="88892462"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3134,7 +3134,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23745984"/>
+        <c:crossAx val="91149792"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3142,7 +3142,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23745984"/>
+        <c:axId val="91149792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="25"/>
@@ -3177,7 +3177,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79773851"/>
+        <c:crossAx val="88892462"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -3270,9 +3270,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -3480,9 +3482,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -3690,9 +3694,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -3900,9 +3906,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -4170,9 +4178,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>24480</xdr:colOff>
+      <xdr:colOff>24120</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>148680</xdr:rowOff>
+      <xdr:rowOff>148320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4181,7 +4189,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6617880" cy="4874760"/>
+        <a:ext cx="6617520" cy="4874400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4200,9 +4208,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884160</xdr:colOff>
+      <xdr:colOff>883800</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4211,7 +4219,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5002560" cy="2769840"/>
+        <a:ext cx="5002200" cy="2769480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4235,9 +4243,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>34200</xdr:colOff>
+      <xdr:colOff>33840</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>148680</xdr:rowOff>
+      <xdr:rowOff>148320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4246,7 +4254,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5899680" y="38160"/>
-        <a:ext cx="6627600" cy="4874760"/>
+        <a:ext cx="6627240" cy="4874400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4265,9 +4273,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>884160</xdr:colOff>
+      <xdr:colOff>883800</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4276,7 +4284,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="762120" y="2209680"/>
-        <a:ext cx="5002560" cy="2769840"/>
+        <a:ext cx="5002200" cy="2769480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>